<commit_message>
chore(preview): OR.PA outputs regeneres
</commit_message>
<xml_diff>
--- a/preview/OR.PA/OR.PA_financials.xlsx
+++ b/preview/OR.PA/OR.PA_financials.xlsx
@@ -8055,10 +8055,18 @@
         </is>
       </c>
       <c r="D29" s="266" t="n"/>
-      <c r="E29" s="266" t="n"/>
-      <c r="F29" s="266" t="n"/>
-      <c r="G29" s="266" t="n"/>
-      <c r="H29" s="266" t="n"/>
+      <c r="E29" s="266" t="n">
+        <v>-502.3</v>
+      </c>
+      <c r="F29" s="266" t="n">
+        <v>-503.3</v>
+      </c>
+      <c r="G29" s="266" t="n">
+        <v>-497.5</v>
+      </c>
+      <c r="H29" s="266" t="n">
+        <v>-501.5</v>
+      </c>
     </row>
     <row r="30" ht="15" customHeight="1">
       <c r="A30" s="3" t="n"/>
@@ -9095,10 +9103,18 @@
         </is>
       </c>
       <c r="D79" s="266" t="n"/>
-      <c r="E79" s="266" t="n"/>
-      <c r="F79" s="266" t="n"/>
-      <c r="G79" s="266" t="n"/>
-      <c r="H79" s="266" t="n"/>
+      <c r="E79" s="266" t="n">
+        <v>-142.8</v>
+      </c>
+      <c r="F79" s="266" t="n">
+        <v>-170.7</v>
+      </c>
+      <c r="G79" s="266" t="n">
+        <v>-1927</v>
+      </c>
+      <c r="H79" s="266" t="n">
+        <v>2509</v>
+      </c>
     </row>
     <row r="80" ht="15" customHeight="1" thickBot="1">
       <c r="A80" s="3" t="n"/>

</xml_diff>